<commit_message>
Cap nhat file excel
</commit_message>
<xml_diff>
--- a/tên các tỉnh.xlsx
+++ b/tên các tỉnh.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MyPC\Desktop\KHKT 2027\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="13890"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="16608" windowHeight="9432"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="144525"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -174,9 +168,6 @@
     <t>Đắk Nông, Lâm Đồng, Bình Thuận</t>
   </si>
   <si>
-    <t>Đồng Nai</t>
-  </si>
-  <si>
     <t>Bình Phước, Đồng Nai</t>
   </si>
   <si>
@@ -227,7 +218,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -237,7 +228,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -249,7 +240,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -259,7 +250,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -272,7 +263,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -282,7 +273,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -294,7 +285,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -304,7 +295,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -317,7 +308,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -327,7 +318,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -339,7 +330,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -349,7 +340,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -362,7 +353,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -372,7 +363,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -384,7 +375,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -394,7 +385,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -407,7 +398,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -417,7 +408,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -429,7 +420,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -439,7 +430,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -452,7 +443,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -462,7 +453,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -474,7 +465,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -484,7 +475,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -497,7 +488,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -507,7 +498,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -519,7 +510,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -529,7 +520,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -542,7 +533,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -552,7 +543,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -564,7 +555,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -574,7 +565,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -587,7 +578,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -597,7 +588,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -609,7 +600,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -619,7 +610,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -632,7 +623,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -642,7 +633,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -654,7 +645,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -664,7 +655,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -677,7 +668,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -687,7 +678,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -699,7 +690,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -709,7 +700,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -721,7 +712,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -731,7 +722,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -744,7 +735,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -754,7 +745,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -766,7 +757,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -776,7 +767,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -789,7 +780,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -799,7 +790,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -810,7 +801,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -821,7 +812,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -832,7 +823,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -843,7 +834,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -856,7 +847,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -866,7 +857,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -878,7 +869,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -888,7 +879,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -901,7 +892,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -911,7 +902,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -923,7 +914,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -933,7 +924,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -946,7 +937,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -956,7 +947,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -968,7 +959,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -978,7 +969,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -991,7 +982,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1001,7 +992,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1013,7 +1004,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1023,7 +1014,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1036,7 +1027,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1046,7 +1037,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1058,7 +1049,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1068,7 +1059,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1081,7 +1072,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1091,7 +1082,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1103,7 +1094,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1113,7 +1104,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1125,7 +1116,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1135,7 +1126,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1148,7 +1139,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1158,7 +1149,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1170,7 +1161,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1180,7 +1171,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1193,7 +1184,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1203,7 +1194,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1215,7 +1206,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1225,7 +1216,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1236,7 +1227,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1247,7 +1238,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1260,7 +1251,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1270,7 +1261,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1282,7 +1273,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1292,7 +1283,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1304,7 +1295,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1314,7 +1305,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1327,7 +1318,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1337,7 +1328,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1349,7 +1340,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1359,7 +1350,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1372,7 +1363,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1382,7 +1373,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1394,7 +1385,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1404,7 +1395,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1417,7 +1408,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1427,7 +1418,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1439,7 +1430,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1449,7 +1440,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1461,7 +1452,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1471,7 +1462,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1484,7 +1475,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1494,7 +1485,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1506,7 +1497,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1516,7 +1507,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1528,7 +1519,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1538,7 +1529,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1551,7 +1542,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1561,7 +1552,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1573,7 +1564,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1583,7 +1574,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1596,7 +1587,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1606,7 +1597,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1618,7 +1609,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1628,7 +1619,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1640,7 +1631,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1650,7 +1641,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1663,7 +1654,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1673,7 +1664,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1685,7 +1676,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1695,7 +1686,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1708,7 +1699,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1718,7 +1709,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1730,7 +1721,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1740,7 +1731,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1752,7 +1743,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1762,7 +1753,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1775,7 +1766,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1785,7 +1776,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1797,7 +1788,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1807,7 +1798,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1820,7 +1811,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1830,7 +1821,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1842,7 +1833,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1852,7 +1843,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1865,7 +1856,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1875,7 +1866,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1887,7 +1878,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1897,7 +1888,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1910,7 +1901,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1920,7 +1911,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1932,7 +1923,7 @@
         <b/>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -1942,7 +1933,7 @@
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
-        <rFont val="Times New Roman"/>
+        <rFont val="Calibri Light"/>
         <family val="1"/>
         <scheme val="major"/>
       </rPr>
@@ -3024,24 +3015,12 @@
 Điểm nổi bật: Phòng làm việc của Tổng thống Việt Nam Cộng hòa, hầm chỉ huy, xe tăng 390 và kiến trúc hiện đại.</t>
   </si>
   <si>
-    <t>2. Khu du lịch Đại Nam (Bình Dương)
-Loại: Khu du lịch tổng hợp.
-Mô tả: Đại Nam là một trong những khu du lịch lớn nhất Việt Nam với nhiều hạng mục như đền thờ, biển nhân tạo, vườn thú mở và khu vui chơi giải trí.
-Điểm nổi bật: Biển nhân tạo, vườn thú safari, trường đua và các trò chơi cảm giác mạnh.</t>
-  </si>
-  <si>
     <t>4. Bãi Sau Vũng Tàu (Bà Rịa - Vũng Tàu)
 Loại: Khu du lịch biển.
 Mô tả: Bãi Sau là bãi biển nổi tiếng nhất của thành phố Vũng Tàu với bãi cát dài, nước biển sạch và nhiều khu nghỉ dưỡng, khách sạn.
 Điểm nổi bật: Tắm biển, dạo bộ ven biển, thưởng thức hải sản và ngắm bình minh.</t>
   </si>
   <si>
-    <t>3. Nhà tù Côn Đảo (Bà Rịa - Vũng Tàu)
-Loại: Di tích lịch sử quốc gia đặc biệt.
-Mô tả: Nhà tù Côn Đảo là hệ thống nhà giam do thực dân Pháp và đế quốc Mỹ xây dựng để giam giữ các chiến sĩ cách mạng. Đây là một trong những di tích lịch sử quan trọng của Việt Nam.
-Điểm nổi bật: Chuồng cọp Côn Đảo, nghĩa trang Hàng Dương và các khu trưng bày lịch sử.</t>
-  </si>
-  <si>
     <t>https://drive.google.com/file/d/1ncdsvGsVYhro1iWTRCeekrsC1hTVR9q6/view?usp=sharing</t>
   </si>
   <si>
@@ -3632,23 +3611,38 @@
   <si>
     <t>https://www.google.com/maps/search/?api=1&amp;query=H%C3%B2n+%C4%90%C3%A1+B%E1%BA%A1c%2C+Tr%E1%BA%A7n+V%C4%83n+Th%E1%BB%9Di%2C+C%C3%A0+Mau&amp;utm_source=chatgpt.com</t>
   </si>
+  <si>
+    <t>TP. Đồng Nai</t>
+  </si>
+  <si>
+    <t>3. Nhà tù Côn Đảo
+Loại: Di tích lịch sử quốc gia đặc biệt.
+Mô tả: Nhà tù Côn Đảo là hệ thống nhà giam do thực dân Pháp và đế quốc Mỹ xây dựng để giam giữ các chiến sĩ cách mạng. Đây là một trong những di tích lịch sử quan trọng của Việt Nam.
+Điểm nổi bật: Chuồng cọp Côn Đảo, nghĩa trang Hàng Dương và các khu trưng bày lịch sử.</t>
+  </si>
+  <si>
+    <t>2. Khu du lịch Đại Nam 
+Loại: Khu du lịch tổng hợp.
+Mô tả: Đại Nam là một trong những khu du lịch lớn nhất Việt Nam với nhiều hạng mục như đền thờ, biển nhân tạo, vườn thú mở và khu vui chơi giải trí.
+Điểm nổi bật: Biển nhân tạo, vườn thú safari, trường đua và các trò chơi cảm giác mạnh.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
+      <name val="Calibri Light"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
@@ -3656,14 +3650,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
+      <name val="Calibri Light"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
+      <name val="Calibri Light"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
@@ -3671,7 +3665,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Times New Roman"/>
+      <name val="Calibri Light"/>
       <family val="1"/>
       <scheme val="major"/>
     </font>
@@ -3679,7 +3673,7 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -3818,7 +3812,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -3870,7 +3864,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -4064,7 +4058,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4073,18 +4067,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H137"/>
-  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="12.109375" style="3" customWidth="1"/>
     <col min="2" max="2" width="23" style="3" customWidth="1"/>
-    <col min="3" max="3" width="56.75" style="14" customWidth="1"/>
-    <col min="4" max="4" width="79.625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="83.375" style="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="180.5" style="14" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.75" style="3"/>
+    <col min="3" max="3" width="56.77734375" style="14" customWidth="1"/>
+    <col min="4" max="4" width="79.6640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="83.33203125" style="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="180.44140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.77734375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="61.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="61.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -4098,13 +4092,13 @@
         <v>3</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
         <v>4</v>
       </c>
@@ -4112,61 +4106,61 @@
         <v>5</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="93" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17"/>
       <c r="B3" s="17"/>
       <c r="C3" s="18"/>
       <c r="D3" s="11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="78" customHeight="1" x14ac:dyDescent="0.25">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="78" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="17"/>
       <c r="B4" s="17"/>
       <c r="C4" s="18"/>
       <c r="D4" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="17"/>
       <c r="B5" s="17"/>
       <c r="C5" s="18"/>
       <c r="D5" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="105" x14ac:dyDescent="0.25">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" s="17" t="s">
         <v>6</v>
       </c>
@@ -4174,62 +4168,62 @@
         <v>6</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="109.15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="109.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="17"/>
       <c r="B7" s="17"/>
       <c r="C7" s="18"/>
       <c r="D7" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="95.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="95.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="18"/>
       <c r="D8" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="101.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="101.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="17"/>
       <c r="B9" s="17"/>
       <c r="C9" s="18"/>
       <c r="D9" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="H9" s="7"/>
     </row>
-    <row r="10" spans="1:8" ht="101.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="101.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
         <v>7</v>
       </c>
@@ -4237,64 +4231,64 @@
         <v>7</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="H10" s="7"/>
     </row>
-    <row r="11" spans="1:8" ht="101.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="101.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="17"/>
       <c r="B11" s="17"/>
       <c r="C11" s="18"/>
       <c r="D11" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="H11" s="7"/>
     </row>
-    <row r="12" spans="1:8" ht="86.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="17"/>
       <c r="B12" s="17"/>
       <c r="C12" s="18"/>
       <c r="D12" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="H12" s="7"/>
     </row>
-    <row r="13" spans="1:8" ht="92.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="92.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="17"/>
       <c r="B13" s="17"/>
       <c r="C13" s="18"/>
       <c r="D13" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="92.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="92.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="17" t="s">
         <v>8</v>
       </c>
@@ -4302,61 +4296,61 @@
         <v>9</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="92.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="92.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="17"/>
       <c r="B15" s="17"/>
       <c r="C15" s="18"/>
       <c r="D15" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="79.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="79.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="17"/>
       <c r="B16" s="17"/>
       <c r="C16" s="18"/>
       <c r="D16" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="124.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="124.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="17"/>
       <c r="B17" s="17"/>
       <c r="C17" s="18"/>
       <c r="D17" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="124.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="124.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="17" t="s">
         <v>10</v>
       </c>
@@ -4364,103 +4358,103 @@
         <v>11</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="124.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="124.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="17"/>
       <c r="B19" s="17"/>
       <c r="C19" s="18"/>
       <c r="D19" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="124.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="124.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="17"/>
       <c r="B20" s="17"/>
       <c r="C20" s="18"/>
       <c r="D20" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A21" s="17"/>
       <c r="B21" s="17"/>
       <c r="C21" s="18"/>
       <c r="D21" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="11"/>
       <c r="D22" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="11"/>
       <c r="D23" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E23" s="13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="67.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="67.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="11"/>
       <c r="D24" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>12</v>
       </c>
@@ -4468,19 +4462,19 @@
         <v>12</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="17" t="s">
         <v>13</v>
       </c>
@@ -4488,61 +4482,61 @@
         <v>13</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.25">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="17"/>
       <c r="B27" s="17"/>
       <c r="C27" s="18"/>
       <c r="D27" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="85.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="85.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="17"/>
       <c r="B28" s="17"/>
       <c r="C28" s="18"/>
       <c r="D28" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="91.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="91.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="17"/>
       <c r="B29" s="17"/>
       <c r="C29" s="18"/>
       <c r="D29" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="91.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="91.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="17" t="s">
         <v>14</v>
       </c>
@@ -4550,61 +4544,61 @@
         <v>14</v>
       </c>
       <c r="C30" s="18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="91.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="91.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="17"/>
       <c r="B31" s="17"/>
       <c r="C31" s="18"/>
       <c r="D31" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="91.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="91.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="17"/>
       <c r="B32" s="17"/>
       <c r="C32" s="18"/>
       <c r="D32" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" ht="92.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="92.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="17"/>
       <c r="B33" s="17"/>
       <c r="C33" s="18"/>
       <c r="D33" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="92.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="92.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="17" t="s">
         <v>15</v>
       </c>
@@ -4612,61 +4606,61 @@
         <v>16</v>
       </c>
       <c r="C34" s="18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="92.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="92.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="17"/>
       <c r="B35" s="17"/>
       <c r="C35" s="18"/>
       <c r="D35" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="79.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="79.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="17"/>
       <c r="B36" s="17"/>
       <c r="C36" s="18"/>
       <c r="D36" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="93" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="17"/>
       <c r="B37" s="17"/>
       <c r="C37" s="18"/>
       <c r="D37" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="93" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="17" t="s">
         <v>17</v>
       </c>
@@ -4674,61 +4668,61 @@
         <v>18</v>
       </c>
       <c r="C38" s="18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F38" s="13" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="93" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="17"/>
       <c r="B39" s="17"/>
       <c r="C39" s="18"/>
       <c r="D39" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F39" s="16" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="93" customHeight="1" x14ac:dyDescent="0.25">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="93" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="17"/>
       <c r="B40" s="17"/>
       <c r="C40" s="18"/>
       <c r="D40" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F40" s="13" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="118.15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="118.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="17"/>
       <c r="B41" s="17"/>
       <c r="C41" s="18"/>
       <c r="D41" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="118.15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="118.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="17" t="s">
         <v>19</v>
       </c>
@@ -4736,61 +4730,61 @@
         <v>19</v>
       </c>
       <c r="C42" s="18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F42" s="13" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="17"/>
       <c r="B43" s="17"/>
       <c r="C43" s="18"/>
       <c r="D43" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="105" customHeight="1" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="105" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="17"/>
       <c r="B44" s="17"/>
       <c r="C44" s="18"/>
       <c r="D44" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F44" s="13" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="91.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="91.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="17"/>
       <c r="B45" s="17"/>
       <c r="C45" s="18"/>
       <c r="D45" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E45" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="91.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="91.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="17" t="s">
         <v>20</v>
       </c>
@@ -4798,61 +4792,61 @@
         <v>20</v>
       </c>
       <c r="C46" s="18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F46" s="13" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="91.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="91.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="17"/>
       <c r="B47" s="17"/>
       <c r="C47" s="18"/>
       <c r="D47" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F47" s="13" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="91.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="91.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="17"/>
       <c r="B48" s="17"/>
       <c r="C48" s="18"/>
       <c r="D48" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E48" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F48" s="13" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" ht="130.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="130.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="17"/>
       <c r="B49" s="17"/>
       <c r="C49" s="18"/>
       <c r="D49" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F49" s="13" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" ht="130.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" ht="130.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="17" t="s">
         <v>21</v>
       </c>
@@ -4860,61 +4854,61 @@
         <v>22</v>
       </c>
       <c r="C50" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E50" s="13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F50" s="13" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" ht="130.9" customHeight="1" x14ac:dyDescent="0.25">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="130.94999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="17"/>
       <c r="B51" s="17"/>
       <c r="C51" s="18"/>
       <c r="D51" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F51" s="13" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" ht="93.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="17"/>
       <c r="B52" s="17"/>
       <c r="C52" s="18"/>
       <c r="D52" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F52" s="13" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" ht="114.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="114.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="17"/>
       <c r="B53" s="17"/>
       <c r="C53" s="18"/>
       <c r="D53" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E53" s="13" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F53" s="13" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" ht="114.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="114.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="17" t="s">
         <v>23</v>
       </c>
@@ -4922,61 +4916,61 @@
         <v>24</v>
       </c>
       <c r="C54" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E54" s="13" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F54" s="13" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" ht="114.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="114.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="17"/>
       <c r="B55" s="17"/>
       <c r="C55" s="18"/>
       <c r="D55" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E55" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F55" s="13" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" ht="114.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="114.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="17"/>
       <c r="B56" s="17"/>
       <c r="C56" s="18"/>
       <c r="D56" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E56" s="13" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F56" s="13" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" ht="119.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" ht="119.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="17"/>
       <c r="B57" s="17"/>
       <c r="C57" s="18"/>
       <c r="D57" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E57" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F57" s="13" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" ht="119.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" ht="119.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="17" t="s">
         <v>25</v>
       </c>
@@ -4984,61 +4978,61 @@
         <v>26</v>
       </c>
       <c r="C58" s="18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E58" s="13" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F58" s="13" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" ht="119.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="119.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="17"/>
       <c r="B59" s="17"/>
       <c r="C59" s="18"/>
       <c r="D59" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E59" s="13" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F59" s="13" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" ht="119.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="119.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="17"/>
       <c r="B60" s="17"/>
       <c r="C60" s="18"/>
       <c r="D60" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E60" s="13" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F60" s="13" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" ht="113.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="113.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="17"/>
       <c r="B61" s="17"/>
       <c r="C61" s="18"/>
       <c r="D61" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E61" s="13" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F61" s="13" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" ht="113.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="113.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="17" t="s">
         <v>27</v>
       </c>
@@ -5046,61 +5040,61 @@
         <v>27</v>
       </c>
       <c r="C62" s="18" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E62" s="13" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F62" s="13" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" ht="113.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="113.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="17"/>
       <c r="B63" s="17"/>
       <c r="C63" s="18"/>
       <c r="D63" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E63" s="13" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F63" s="13" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" ht="113.45" customHeight="1" x14ac:dyDescent="0.25">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="113.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="17"/>
       <c r="B64" s="17"/>
       <c r="C64" s="18"/>
       <c r="D64" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E64" s="13" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F64" s="13" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A65" s="17"/>
       <c r="B65" s="17"/>
       <c r="C65" s="18"/>
       <c r="D65" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E65" s="13" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F65" s="13" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A66" s="17" t="s">
         <v>28</v>
       </c>
@@ -5108,61 +5102,61 @@
         <v>28</v>
       </c>
       <c r="C66" s="18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E66" s="13" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F66" s="13" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A67" s="17"/>
       <c r="B67" s="17"/>
       <c r="C67" s="18"/>
       <c r="D67" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E67" s="13" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F67" s="13" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A68" s="17"/>
       <c r="B68" s="17"/>
       <c r="C68" s="18"/>
       <c r="D68" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E68" s="13" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F68" s="13" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A69" s="17"/>
       <c r="B69" s="17"/>
       <c r="C69" s="18"/>
       <c r="D69" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E69" s="13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F69" s="13" t="s">
-        <v>437</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" ht="120" x14ac:dyDescent="0.25">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A70" s="17" t="s">
         <v>29</v>
       </c>
@@ -5170,61 +5164,61 @@
         <v>29</v>
       </c>
       <c r="C70" s="18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E70" s="13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F70" s="13" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A71" s="17"/>
       <c r="B71" s="17"/>
       <c r="C71" s="18"/>
       <c r="D71" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E71" s="13" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F71" s="13" t="s">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A72" s="17"/>
       <c r="B72" s="17"/>
       <c r="C72" s="18"/>
       <c r="D72" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E72" s="13" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F72" s="13" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" ht="135" x14ac:dyDescent="0.25">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A73" s="17"/>
       <c r="B73" s="17"/>
       <c r="C73" s="18"/>
       <c r="D73" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E73" s="13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F73" s="13" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A74" s="17" t="s">
         <v>30</v>
       </c>
@@ -5232,61 +5226,61 @@
         <v>31</v>
       </c>
       <c r="C74" s="18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E74" s="13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F74" s="13" t="s">
-        <v>442</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A75" s="17"/>
       <c r="B75" s="17"/>
       <c r="C75" s="18"/>
       <c r="D75" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E75" s="13" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F75" s="13" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A76" s="17"/>
       <c r="B76" s="17"/>
       <c r="C76" s="18"/>
       <c r="D76" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E76" s="13" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F76" s="13" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A77" s="17"/>
       <c r="B77" s="17"/>
       <c r="C77" s="18"/>
       <c r="D77" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E77" s="13" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F77" s="13" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A78" s="17" t="s">
         <v>32</v>
       </c>
@@ -5294,61 +5288,61 @@
         <v>33</v>
       </c>
       <c r="C78" s="18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E78" s="13" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F78" s="13" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A79" s="17"/>
       <c r="B79" s="17"/>
       <c r="C79" s="18"/>
       <c r="D79" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F79" s="13" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A80" s="17"/>
       <c r="B80" s="17"/>
       <c r="C80" s="18"/>
       <c r="D80" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E80" s="13" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F80" s="13" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" ht="120" x14ac:dyDescent="0.25">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A81" s="17"/>
       <c r="B81" s="17"/>
       <c r="C81" s="18"/>
       <c r="D81" s="1" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E81" s="13" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F81" s="13" t="s">
-        <v>449</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" ht="114.75" x14ac:dyDescent="0.25">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A82" s="17" t="s">
         <v>34</v>
       </c>
@@ -5356,61 +5350,61 @@
         <v>35</v>
       </c>
       <c r="C82" s="18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E82" s="15" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F82" s="15" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A83" s="17"/>
       <c r="B83" s="17"/>
       <c r="C83" s="18"/>
       <c r="D83" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E83" s="7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F83" s="7" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A84" s="17"/>
       <c r="B84" s="17"/>
       <c r="C84" s="18"/>
       <c r="D84" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F84" s="13" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A85" s="17"/>
       <c r="B85" s="17"/>
       <c r="C85" s="18"/>
       <c r="D85" s="1" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E85" s="13" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F85" s="13" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A86" s="17" t="s">
         <v>36</v>
       </c>
@@ -5418,61 +5412,61 @@
         <v>37</v>
       </c>
       <c r="C86" s="18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E86" s="13" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F86" s="13" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A87" s="17"/>
       <c r="B87" s="17"/>
       <c r="C87" s="18"/>
       <c r="D87" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E87" s="13" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F87" s="13" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A88" s="17"/>
       <c r="B88" s="17"/>
       <c r="C88" s="18"/>
       <c r="D88" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E88" s="13" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F88" s="13" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A89" s="17"/>
       <c r="B89" s="17"/>
       <c r="C89" s="18"/>
       <c r="D89" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E89" s="13" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F89" s="13" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" ht="120" x14ac:dyDescent="0.25">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A90" s="17" t="s">
         <v>38</v>
       </c>
@@ -5481,60 +5475,60 @@
       </c>
       <c r="C90" s="11"/>
       <c r="D90" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E90" s="13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F90" s="13" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A91" s="17"/>
       <c r="B91" s="17"/>
       <c r="C91" s="18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E91" s="13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F91" s="13" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A92" s="17"/>
       <c r="B92" s="17"/>
       <c r="C92" s="18"/>
       <c r="D92" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E92" s="13" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F92" s="13" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A93" s="17"/>
       <c r="B93" s="17"/>
       <c r="C93" s="18"/>
       <c r="D93" s="1" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E93" s="13" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F93" s="13" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A94" s="17" t="s">
         <v>40</v>
       </c>
@@ -5542,61 +5536,61 @@
         <v>41</v>
       </c>
       <c r="C94" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E94" s="13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F94" s="13" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A95" s="17"/>
       <c r="B95" s="17"/>
       <c r="C95" s="18"/>
       <c r="D95" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E95" s="13" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F95" s="13" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A96" s="17"/>
       <c r="B96" s="17"/>
       <c r="C96" s="18"/>
       <c r="D96" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E96" s="13" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F96" s="13" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A97" s="17"/>
       <c r="B97" s="17"/>
       <c r="C97" s="18"/>
       <c r="D97" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E97" s="13" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F97" s="13" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A98" s="17" t="s">
         <v>42</v>
       </c>
@@ -5604,61 +5598,61 @@
         <v>43</v>
       </c>
       <c r="C98" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E98" s="13" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F98" s="13" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A99" s="17"/>
       <c r="B99" s="17"/>
       <c r="C99" s="18"/>
       <c r="D99" s="1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E99" s="13" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F99" s="13" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A100" s="17"/>
       <c r="B100" s="17"/>
       <c r="C100" s="18"/>
       <c r="D100" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E100" s="13" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F100" s="13" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A101" s="17"/>
       <c r="B101" s="17"/>
       <c r="C101" s="18"/>
       <c r="D101" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E101" s="13" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F101" s="13" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A102" s="17" t="s">
         <v>44</v>
       </c>
@@ -5666,570 +5660,630 @@
         <v>45</v>
       </c>
       <c r="C102" s="18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E102" s="13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F102" s="13" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" ht="270" x14ac:dyDescent="0.25">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A103" s="17"/>
       <c r="B103" s="17"/>
       <c r="C103" s="18"/>
       <c r="D103" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="E103" s="13" t="s">
         <v>306</v>
       </c>
-      <c r="E103" s="13" t="s">
-        <v>307</v>
-      </c>
       <c r="F103" s="13" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A104" s="17"/>
       <c r="B104" s="17"/>
       <c r="C104" s="18"/>
       <c r="D104" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E104" s="13" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F104" s="13" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A105" s="17"/>
       <c r="B105" s="17"/>
       <c r="C105" s="18"/>
       <c r="D105" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="E105" s="13" t="s">
+        <v>308</v>
+      </c>
+      <c r="F105" s="13" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A106" s="17" t="s">
+        <v>503</v>
+      </c>
+      <c r="B106" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="C106" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="D106" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="E105" s="13" t="s">
-        <v>309</v>
-      </c>
-      <c r="F105" s="13" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" ht="105" x14ac:dyDescent="0.25">
-      <c r="A106" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="B106" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="C106" s="18" t="s">
-        <v>95</v>
-      </c>
-      <c r="D106" s="1" t="s">
-        <v>312</v>
-      </c>
       <c r="E106" s="13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F106" s="13" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A107" s="17"/>
       <c r="B107" s="17"/>
       <c r="C107" s="18"/>
       <c r="D107" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E107" s="13" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F107" s="13" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A108" s="17"/>
       <c r="B108" s="17"/>
       <c r="C108" s="18"/>
       <c r="D108" s="1" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E108" s="13" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F108" s="13" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A109" s="17"/>
       <c r="B109" s="17"/>
       <c r="C109" s="18"/>
       <c r="D109" s="1" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E109" s="13" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F109" s="13" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A110" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B110" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="B110" s="17" t="s">
-        <v>49</v>
-      </c>
       <c r="C110" s="18" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E110" s="13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F110" s="13" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A111" s="17"/>
       <c r="B111" s="17"/>
       <c r="C111" s="18"/>
       <c r="D111" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="E111" s="13" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="F111" s="13" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A112" s="17"/>
       <c r="B112" s="17"/>
       <c r="C112" s="18"/>
       <c r="D112" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="E112" s="13" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F112" s="13" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A113" s="17"/>
       <c r="B113" s="17"/>
       <c r="C113" s="18"/>
       <c r="D113" s="1" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="E113" s="13" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="F113" s="13" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" ht="96.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B114" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B114" s="17" t="s">
-        <v>51</v>
-      </c>
       <c r="C114" s="18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E114" s="13" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="F114" s="13" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A115" s="17"/>
       <c r="B115" s="17"/>
       <c r="C115" s="18"/>
       <c r="D115" s="1" t="s">
-        <v>327</v>
+        <v>505</v>
       </c>
       <c r="E115" s="13" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="F115" s="13" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A116" s="17"/>
       <c r="B116" s="17"/>
       <c r="C116" s="18"/>
       <c r="D116" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="E116" s="13" t="s">
         <v>329</v>
       </c>
-      <c r="E116" s="13" t="s">
-        <v>332</v>
-      </c>
       <c r="F116" s="13" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" ht="105.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="17"/>
       <c r="B117" s="17"/>
       <c r="C117" s="18"/>
       <c r="D117" s="1" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="E117" s="13" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="F117" s="13" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" ht="105.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="B118" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="B118" s="17" t="s">
-        <v>53</v>
-      </c>
       <c r="C118" s="18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D118" s="1" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="E118" s="13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F118" s="13" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" ht="105.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="17"/>
       <c r="B119" s="17"/>
       <c r="C119" s="18"/>
       <c r="D119" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="E119" s="13" t="s">
         <v>335</v>
       </c>
-      <c r="E119" s="13" t="s">
-        <v>338</v>
-      </c>
       <c r="F119" s="13" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" ht="105.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="17"/>
       <c r="B120" s="17"/>
       <c r="C120" s="18"/>
       <c r="D120" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="E120" s="7" t="s">
         <v>337</v>
       </c>
-      <c r="E120" s="7" t="s">
-        <v>340</v>
-      </c>
       <c r="F120" s="7" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" ht="120" x14ac:dyDescent="0.25">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A121" s="17"/>
       <c r="B121" s="17"/>
       <c r="C121" s="18"/>
       <c r="D121" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="E121" s="13" t="s">
         <v>336</v>
       </c>
-      <c r="E121" s="13" t="s">
-        <v>339</v>
-      </c>
       <c r="F121" s="13" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A122" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B122" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B122" s="17" t="s">
-        <v>55</v>
-      </c>
       <c r="C122" s="18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="E122" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F122" s="13" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A123" s="17"/>
       <c r="B123" s="17"/>
       <c r="C123" s="18"/>
       <c r="D123" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="E123" s="13" t="s">
         <v>342</v>
       </c>
-      <c r="E123" s="13" t="s">
-        <v>345</v>
-      </c>
       <c r="F123" s="13" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A124" s="17"/>
       <c r="B124" s="17"/>
       <c r="C124" s="18"/>
       <c r="D124" s="1" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="E124" s="13" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="F124" s="13" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A125" s="17"/>
       <c r="B125" s="17"/>
       <c r="C125" s="18"/>
       <c r="D125" s="1" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="E125" s="13" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="F125" s="13" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A126" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="B126" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="B126" s="17" t="s">
-        <v>57</v>
-      </c>
       <c r="C126" s="18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="E126" s="13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F126" s="13" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A127" s="17"/>
       <c r="B127" s="17"/>
       <c r="C127" s="18"/>
       <c r="D127" s="1" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="E127" s="7" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="F127" s="7" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A128" s="17"/>
       <c r="B128" s="17"/>
       <c r="C128" s="18"/>
       <c r="D128" s="1" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="E128" s="13" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="F128" s="13" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A129" s="17"/>
       <c r="B129" s="17"/>
       <c r="C129" s="18"/>
       <c r="D129" s="1" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="E129" s="13" t="s">
+        <v>349</v>
+      </c>
+      <c r="F129" s="13" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A130" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B130" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="C130" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="D130" s="1" t="s">
         <v>352</v>
       </c>
-      <c r="F129" s="13" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" ht="105" x14ac:dyDescent="0.25">
-      <c r="A130" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="B130" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="C130" s="18" t="s">
-        <v>93</v>
-      </c>
-      <c r="D130" s="1" t="s">
-        <v>355</v>
-      </c>
       <c r="E130" s="13" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F130" s="13" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A131" s="17"/>
       <c r="B131" s="17"/>
       <c r="C131" s="18"/>
       <c r="D131" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E131" s="13" t="s">
         <v>356</v>
       </c>
-      <c r="E131" s="13" t="s">
-        <v>359</v>
-      </c>
       <c r="F131" s="13" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A132" s="17"/>
       <c r="B132" s="17"/>
       <c r="C132" s="18"/>
       <c r="D132" s="1" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="E132" s="13" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="F132" s="13" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A133" s="17"/>
       <c r="B133" s="17"/>
       <c r="C133" s="18"/>
       <c r="D133" s="1" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="E133" s="13" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="F133" s="13" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="134" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A134" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B134" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="B134" s="17" t="s">
-        <v>61</v>
-      </c>
       <c r="C134" s="18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="E134" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F134" s="13" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A135" s="17"/>
       <c r="B135" s="17"/>
       <c r="C135" s="18"/>
       <c r="D135" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="E135" s="13" t="s">
         <v>363</v>
       </c>
-      <c r="E135" s="13" t="s">
-        <v>366</v>
-      </c>
       <c r="F135" s="13" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A136" s="17"/>
       <c r="B136" s="17"/>
       <c r="C136" s="18"/>
       <c r="D136" s="1" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="E136" s="13" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="F136" s="13" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A137" s="17"/>
       <c r="B137" s="17"/>
       <c r="C137" s="18"/>
       <c r="D137" s="1" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="E137" s="13" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="F137" s="13" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="99">
-    <mergeCell ref="A130:A133"/>
-    <mergeCell ref="B130:B133"/>
-    <mergeCell ref="C130:C133"/>
-    <mergeCell ref="A134:A137"/>
-    <mergeCell ref="B134:B137"/>
-    <mergeCell ref="C134:C137"/>
-    <mergeCell ref="A122:A125"/>
-    <mergeCell ref="B122:B125"/>
-    <mergeCell ref="C122:C125"/>
-    <mergeCell ref="A126:A129"/>
-    <mergeCell ref="B126:B129"/>
-    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="C14:C17"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="C38:C41"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="C42:C45"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="C50:C53"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="C66:C69"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="C70:C73"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="B74:B77"/>
+    <mergeCell ref="C74:C77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="B78:B81"/>
+    <mergeCell ref="C78:C81"/>
+    <mergeCell ref="A82:A85"/>
+    <mergeCell ref="B82:B85"/>
+    <mergeCell ref="C82:C85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="C86:C89"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="C91:C93"/>
+    <mergeCell ref="A94:A97"/>
+    <mergeCell ref="B94:B97"/>
+    <mergeCell ref="C94:C97"/>
+    <mergeCell ref="A98:A101"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="C98:C101"/>
     <mergeCell ref="A118:A121"/>
     <mergeCell ref="B118:B121"/>
     <mergeCell ref="C118:C121"/>
@@ -6245,78 +6299,18 @@
     <mergeCell ref="C110:C113"/>
     <mergeCell ref="A114:A117"/>
     <mergeCell ref="B114:B117"/>
-    <mergeCell ref="A94:A97"/>
-    <mergeCell ref="B94:B97"/>
-    <mergeCell ref="C94:C97"/>
-    <mergeCell ref="A98:A101"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="C98:C101"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="C86:C89"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="C91:C93"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="B78:B81"/>
-    <mergeCell ref="C78:C81"/>
-    <mergeCell ref="A82:A85"/>
-    <mergeCell ref="B82:B85"/>
-    <mergeCell ref="C82:C85"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="C70:C73"/>
-    <mergeCell ref="A74:A77"/>
-    <mergeCell ref="B74:B77"/>
-    <mergeCell ref="C74:C77"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="C62:C65"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="C66:C69"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="C58:C61"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="C50:C53"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="C38:C41"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="C42:C45"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="C30:C33"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="C18:C21"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="C26:C29"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="C14:C17"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="A122:A125"/>
+    <mergeCell ref="B122:B125"/>
+    <mergeCell ref="C122:C125"/>
+    <mergeCell ref="A126:A129"/>
+    <mergeCell ref="B126:B129"/>
+    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="A130:A133"/>
+    <mergeCell ref="B130:B133"/>
+    <mergeCell ref="C130:C133"/>
+    <mergeCell ref="A134:A137"/>
+    <mergeCell ref="B134:B137"/>
+    <mergeCell ref="C134:C137"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E9" r:id="rId1"/>

</xml_diff>